<commit_message>
Revert strictly to original 25 problem statements and allocate 27 pairs
</commit_message>
<xml_diff>
--- a/Synapse_Teams_Problem_Statements_Updated.xlsx
+++ b/Synapse_Teams_Problem_Statements_Updated.xlsx
@@ -468,13 +468,13 @@
         <v>yathish chandh reddy.P, rishwan abuthakir.j, sri balaji.E</v>
       </c>
       <c r="G2" t="str">
-        <v>PS #16</v>
+        <v>PS #10</v>
       </c>
       <c r="H2" t="str">
-        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
+        <v>Catastrophe Risk Modelling</v>
       </c>
       <c r="I2" t="str">
-        <v>AI Mesh Networks &amp; Disaster Response</v>
+        <v>ClimateTech &amp; Catastrophe Risk</v>
       </c>
       <c r="J2" t="str">
         <v>HARD</v>
@@ -503,13 +503,13 @@
         <v>SHARAN, Divakar R, DHEENA D</v>
       </c>
       <c r="G3" t="str">
-        <v>PS #04</v>
+        <v>PS #05</v>
       </c>
       <c r="H3" t="str">
-        <v>Open Banking &amp; APIs</v>
+        <v>Payments Modernisation</v>
       </c>
       <c r="I3" t="str">
-        <v>Open Banking &amp; API Ecosystems</v>
+        <v>Payments Modernisation</v>
       </c>
       <c r="J3" t="str">
         <v>MEDIUM</v>
@@ -538,19 +538,19 @@
         <v>Deepak M, Gubendhiran M, Gokhulakrishnapriyan K</v>
       </c>
       <c r="G4" t="str">
-        <v>PS #01</v>
+        <v>PS #24</v>
       </c>
       <c r="H4" t="str">
-        <v>Lending &amp; Credit</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="I4" t="str">
-        <v>FinTech &amp; AI</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
       <c r="J4" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K4" t="str">
-        <v>SY29 - WhyNot</v>
+        <v>SY29 - WhyNot | SY53 - Tech Titans | SY54 - Claude Busters</v>
       </c>
     </row>
     <row r="5">
@@ -573,13 +573,13 @@
         <v>SHARU KESAVAN P, SANJEEV RAJ V, THANA G K</v>
       </c>
       <c r="G5" t="str">
-        <v>PS #14</v>
+        <v>PS #02</v>
       </c>
       <c r="H5" t="str">
-        <v>Readmission Prevention</v>
+        <v>Fraud Detection</v>
       </c>
       <c r="I5" t="str">
-        <v>HealthTech &amp; Predictive AI</v>
+        <v>FinTech &amp; Cybersecurity</v>
       </c>
       <c r="J5" t="str">
         <v>HARD</v>
@@ -608,13 +608,13 @@
         <v>Nithya Sri S</v>
       </c>
       <c r="G6" t="str">
-        <v>PS #17</v>
+        <v>PS #19</v>
       </c>
       <c r="H6" t="str">
-        <v>Real-Time Indian Sign Language Translator</v>
+        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
       </c>
       <c r="I6" t="str">
-        <v>Computer Vision &amp; Accessibility (ISL)</v>
+        <v>Enterprise AI &amp; Multi-Source RAG</v>
       </c>
       <c r="J6" t="str">
         <v>HARD</v>
@@ -643,13 +643,13 @@
         <v>Romanya R</v>
       </c>
       <c r="G7" t="str">
-        <v>PS #03</v>
+        <v>PS #04</v>
       </c>
       <c r="H7" t="str">
-        <v>Personalised Banking</v>
+        <v>Open Banking &amp; APIs</v>
       </c>
       <c r="I7" t="str">
-        <v>FinTech &amp; Personalization</v>
+        <v>Open Banking &amp; API Ecosystems</v>
       </c>
       <c r="J7" t="str">
         <v>MEDIUM</v>
@@ -678,13 +678,13 @@
         <v>Ragul G</v>
       </c>
       <c r="G8" t="str">
-        <v>PS #07</v>
+        <v>PS #08</v>
       </c>
       <c r="H8" t="str">
-        <v>End-to-End Claims Automation</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="I8" t="str">
-        <v>InsurTech &amp; Claims Processing</v>
+        <v>InsurTech &amp; IoT Telematics</v>
       </c>
       <c r="J8" t="str">
         <v>MEDIUM</v>
@@ -713,16 +713,16 @@
         <v>Lakshmiram S</v>
       </c>
       <c r="G9" t="str">
-        <v>PS #10</v>
+        <v>PS #25</v>
       </c>
       <c r="H9" t="str">
-        <v>Catastrophe Risk Modelling</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="I9" t="str">
-        <v>ClimateTech &amp; Catastrophe Risk</v>
+        <v>Smart Mobility &amp; Usage-Based Insurance</v>
       </c>
       <c r="J9" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K9" t="str">
         <v>SY34 - TECH NOVA</v>
@@ -783,13 +783,13 @@
         <v>Ragavi M, Nivisri G, pooja G</v>
       </c>
       <c r="G11" t="str">
-        <v>PS #22</v>
+        <v>PS #17</v>
       </c>
       <c r="H11" t="str">
-        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
+        <v>Real-Time Indian Sign Language Translator</v>
       </c>
       <c r="I11" t="str">
-        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
+        <v>Computer Vision &amp; Accessibility (ISL)</v>
       </c>
       <c r="J11" t="str">
         <v>HARD</v>
@@ -818,13 +818,13 @@
         <v>DHARINEESH V, Nill, Nill</v>
       </c>
       <c r="G12" t="str">
-        <v>PS #13</v>
+        <v>PS #18</v>
       </c>
       <c r="H12" t="str">
-        <v>Healthcare Interoperability</v>
+        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
       </c>
       <c r="I12" t="str">
-        <v>HealthTech &amp; FHIR Interoperability</v>
+        <v>LegalTech &amp; Contract Risk Copilot</v>
       </c>
       <c r="J12" t="str">
         <v>HARD</v>
@@ -853,16 +853,16 @@
         <v>Kathirvel T, Kanish M, Kaviraj R</v>
       </c>
       <c r="G13" t="str">
-        <v>PS #27</v>
+        <v>PS #22</v>
       </c>
       <c r="H13" t="str">
-        <v>Multimodal AI Copilot for Accessibility &amp; Assistive Vision</v>
+        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
       </c>
       <c r="I13" t="str">
-        <v>Computer Vision &amp; Assistive AI</v>
+        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
       </c>
       <c r="J13" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K13" t="str">
         <v>SY38 - AKATSUKI</v>
@@ -888,13 +888,13 @@
         <v>Hiwins Daisin A, Likith K</v>
       </c>
       <c r="G14" t="str">
-        <v>PS #24</v>
+        <v>PS #14</v>
       </c>
       <c r="H14" t="str">
-        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
+        <v>Readmission Prevention</v>
       </c>
       <c r="I14" t="str">
-        <v>Digital Forensics &amp; Evidence Integrity</v>
+        <v>HealthTech &amp; Predictive AI</v>
       </c>
       <c r="J14" t="str">
         <v>HARD</v>
@@ -923,16 +923,16 @@
         <v>Kanishka L, Harini V, Durkkadharshini M</v>
       </c>
       <c r="G15" t="str">
-        <v>PS #18</v>
+        <v>PS #09</v>
       </c>
       <c r="H15" t="str">
-        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
+        <v>Embedded Insurance</v>
       </c>
       <c r="I15" t="str">
-        <v>LegalTech &amp; Contract Risk Copilot</v>
+        <v>InsurTech &amp; Embedded Finance</v>
       </c>
       <c r="J15" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K15" t="str">
         <v>SY40 - Code Creepers</v>
@@ -958,16 +958,16 @@
         <v>Deepak PM, Dinesh Karthick R, Arunkumar G</v>
       </c>
       <c r="G16" t="str">
-        <v>PS #11</v>
+        <v>PS #20</v>
       </c>
       <c r="H16" t="str">
-        <v>Prior Authorisation Automation</v>
+        <v>AI Grievance Redressal Prioritization System</v>
       </c>
       <c r="I16" t="str">
-        <v>HealthTech &amp; Prior Authorisation</v>
+        <v>GovTech &amp; Multilingual Grievance NLP</v>
       </c>
       <c r="J16" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K16" t="str">
         <v>SY41 - Team Innovator's</v>
@@ -993,13 +993,13 @@
         <v>Malinie T, Kamali R, Supriya j</v>
       </c>
       <c r="G17" t="str">
-        <v>PS #08</v>
+        <v>PS #12</v>
       </c>
       <c r="H17" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Clinical Documentation</v>
       </c>
       <c r="I17" t="str">
-        <v>InsurTech &amp; IoT Telematics</v>
+        <v>HealthTech &amp; Clinical Speech NLP</v>
       </c>
       <c r="J17" t="str">
         <v>MEDIUM</v>
@@ -1028,13 +1028,13 @@
         <v>Gokulnath S, Dinesh C, Balasubramani P</v>
       </c>
       <c r="G18" t="str">
-        <v>PS #12</v>
+        <v>PS #07</v>
       </c>
       <c r="H18" t="str">
-        <v>Clinical Documentation</v>
+        <v>End-to-End Claims Automation</v>
       </c>
       <c r="I18" t="str">
-        <v>HealthTech &amp; Clinical Speech NLP</v>
+        <v>InsurTech &amp; Claims Processing</v>
       </c>
       <c r="J18" t="str">
         <v>MEDIUM</v>
@@ -1063,16 +1063,16 @@
         <v>Kabilan S, Jerry Mathew . J, Narendran V</v>
       </c>
       <c r="G19" t="str">
-        <v>PS #06</v>
+        <v>PS #03</v>
       </c>
       <c r="H19" t="str">
-        <v>Underwriting Automation</v>
+        <v>Personalised Banking</v>
       </c>
       <c r="I19" t="str">
-        <v>InsurTech &amp; Automated Underwriting</v>
+        <v>FinTech &amp; Personalization</v>
       </c>
       <c r="J19" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K19" t="str">
         <v>SY44 - INNOVEXA</v>
@@ -1098,16 +1098,16 @@
         <v>Magha Sri P</v>
       </c>
       <c r="G20" t="str">
-        <v>PS #26</v>
+        <v>PS #15</v>
       </c>
       <c r="H20" t="str">
-        <v>Autonomous Zero-Trust API Security &amp; Anomaly Shield</v>
+        <v>Value-Based Care Analytics</v>
       </c>
       <c r="I20" t="str">
-        <v>Cybersecurity &amp; Cloud Security</v>
+        <v>HealthTech &amp; Value-Based Analytics</v>
       </c>
       <c r="J20" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K20" t="str">
         <v>SY45 - Neura Nova</v>
@@ -1133,16 +1133,16 @@
         <v>Moulitharan IR, Nithish Rajan P, Nagaraj V</v>
       </c>
       <c r="G21" t="str">
-        <v>PS #20</v>
+        <v>PS #16</v>
       </c>
       <c r="H21" t="str">
-        <v>AI Grievance Redressal Prioritization System</v>
+        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
       </c>
       <c r="I21" t="str">
-        <v>GovTech &amp; Multilingual Grievance NLP</v>
+        <v>AI Mesh Networks &amp; Disaster Response</v>
       </c>
       <c r="J21" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K21" t="str">
         <v>SY46 - Hellfire</v>
@@ -1203,13 +1203,13 @@
         <v>NISHANTH A</v>
       </c>
       <c r="G23" t="str">
-        <v>PS #19</v>
+        <v>PS #13</v>
       </c>
       <c r="H23" t="str">
-        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
+        <v>Healthcare Interoperability</v>
       </c>
       <c r="I23" t="str">
-        <v>Enterprise AI &amp; Multi-Source RAG</v>
+        <v>HealthTech &amp; FHIR Interoperability</v>
       </c>
       <c r="J23" t="str">
         <v>HARD</v>
@@ -1238,16 +1238,16 @@
         <v>Logeshwaran G, Jagan M, Mithun C</v>
       </c>
       <c r="G24" t="str">
-        <v>PS #15</v>
+        <v>PS #06</v>
       </c>
       <c r="H24" t="str">
-        <v>Value-Based Care Analytics</v>
+        <v>Underwriting Automation</v>
       </c>
       <c r="I24" t="str">
-        <v>HealthTech &amp; Value-Based Analytics</v>
+        <v>InsurTech &amp; Automated Underwriting</v>
       </c>
       <c r="J24" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K24" t="str">
         <v>SY49 - AI Assist</v>
@@ -1273,19 +1273,19 @@
         <v>SHRENITHI B, SASMITHA M, SANGAMITHRA K</v>
       </c>
       <c r="G25" t="str">
-        <v>PS #09</v>
+        <v>PS #01</v>
       </c>
       <c r="H25" t="str">
-        <v>Embedded Insurance</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="I25" t="str">
-        <v>InsurTech &amp; Embedded Finance</v>
+        <v>FinTech &amp; AI</v>
       </c>
       <c r="J25" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="K25" t="str">
-        <v>SY50 - Chaos coders</v>
+        <v>SY26 - Phoenix | SY50 - Chaos coders | SY52 - Hack Fusion</v>
       </c>
     </row>
     <row r="26">
@@ -1308,16 +1308,16 @@
         <v>Subiksha S, Sudheksha P, Tharani T</v>
       </c>
       <c r="G26" t="str">
-        <v>PS #25</v>
+        <v>PS #11</v>
       </c>
       <c r="H26" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Prior Authorisation Automation</v>
       </c>
       <c r="I26" t="str">
-        <v>Smart Mobility &amp; Usage-Based Insurance</v>
+        <v>HealthTech &amp; Prior Authorisation</v>
       </c>
       <c r="J26" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K26" t="str">
         <v>SY51 - MindForge</v>
@@ -1343,19 +1343,19 @@
         <v>SARAVANAVEL K, SANTHOSH BALAJI N, KISHORE R</v>
       </c>
       <c r="G27" t="str">
-        <v>PS #02</v>
+        <v>PS #01</v>
       </c>
       <c r="H27" t="str">
-        <v>Fraud Detection</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="I27" t="str">
-        <v>FinTech &amp; Cybersecurity</v>
+        <v>FinTech &amp; AI</v>
       </c>
       <c r="J27" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K27" t="str">
-        <v>SY52 - Hack Fusion</v>
+        <v>SY24 - TECH SPARKZ | SY50 - Chaos coders | SY52 - Hack Fusion</v>
       </c>
     </row>
     <row r="28">
@@ -1378,13 +1378,13 @@
         <v>VISHNUVARDHAN A, THARUN J V, SUHANDHAN K</v>
       </c>
       <c r="G28" t="str">
-        <v>PS #16</v>
+        <v>PS #10</v>
       </c>
       <c r="H28" t="str">
-        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
+        <v>Catastrophe Risk Modelling</v>
       </c>
       <c r="I28" t="str">
-        <v>AI Mesh Networks &amp; Disaster Response</v>
+        <v>ClimateTech &amp; Catastrophe Risk</v>
       </c>
       <c r="J28" t="str">
         <v>HARD</v>
@@ -1413,13 +1413,13 @@
         <v>AAKASH M</v>
       </c>
       <c r="G29" t="str">
-        <v>PS #04</v>
+        <v>PS #05</v>
       </c>
       <c r="H29" t="str">
-        <v>Open Banking &amp; APIs</v>
+        <v>Payments Modernisation</v>
       </c>
       <c r="I29" t="str">
-        <v>Open Banking &amp; API Ecosystems</v>
+        <v>Payments Modernisation</v>
       </c>
       <c r="J29" t="str">
         <v>MEDIUM</v>
@@ -1448,19 +1448,19 @@
         <v>PRIYADHARSHINI B, SHERIN INFANTA, SANTHIYA R</v>
       </c>
       <c r="G30" t="str">
-        <v>PS #01</v>
+        <v>PS #24</v>
       </c>
       <c r="H30" t="str">
-        <v>Lending &amp; Credit</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="I30" t="str">
-        <v>FinTech &amp; AI</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
       <c r="J30" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K30" t="str">
-        <v>SY03 - BroVerse</v>
+        <v>SY03 - BroVerse | SY53 - Tech Titans | SY54 - Claude Busters</v>
       </c>
     </row>
     <row r="31">
@@ -1483,13 +1483,13 @@
         <v>Reyas B, Santhosh M, Sudeep</v>
       </c>
       <c r="G31" t="str">
-        <v>PS #14</v>
+        <v>PS #02</v>
       </c>
       <c r="H31" t="str">
-        <v>Readmission Prevention</v>
+        <v>Fraud Detection</v>
       </c>
       <c r="I31" t="str">
-        <v>HealthTech &amp; Predictive AI</v>
+        <v>FinTech &amp; Cybersecurity</v>
       </c>
       <c r="J31" t="str">
         <v>HARD</v>
@@ -1518,13 +1518,13 @@
         <v>K.Sanjay, P.Rafeal nadal, K.S.Sachin</v>
       </c>
       <c r="G32" t="str">
-        <v>PS #17</v>
+        <v>PS #19</v>
       </c>
       <c r="H32" t="str">
-        <v>Real-Time Indian Sign Language Translator</v>
+        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
       </c>
       <c r="I32" t="str">
-        <v>Computer Vision &amp; Accessibility (ISL)</v>
+        <v>Enterprise AI &amp; Multi-Source RAG</v>
       </c>
       <c r="J32" t="str">
         <v>HARD</v>
@@ -1553,13 +1553,13 @@
         <v>Mithun T. G, Mohammed shuaif. S, Methilesh. R</v>
       </c>
       <c r="G33" t="str">
-        <v>PS #03</v>
+        <v>PS #04</v>
       </c>
       <c r="H33" t="str">
-        <v>Personalised Banking</v>
+        <v>Open Banking &amp; APIs</v>
       </c>
       <c r="I33" t="str">
-        <v>FinTech &amp; Personalization</v>
+        <v>Open Banking &amp; API Ecosystems</v>
       </c>
       <c r="J33" t="str">
         <v>MEDIUM</v>
@@ -1588,13 +1588,13 @@
         <v>Nikitha K, Kowsalya B, Meera B</v>
       </c>
       <c r="G34" t="str">
-        <v>PS #07</v>
+        <v>PS #08</v>
       </c>
       <c r="H34" t="str">
-        <v>End-to-End Claims Automation</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="I34" t="str">
-        <v>InsurTech &amp; Claims Processing</v>
+        <v>InsurTech &amp; IoT Telematics</v>
       </c>
       <c r="J34" t="str">
         <v>MEDIUM</v>
@@ -1623,16 +1623,16 @@
         <v>MANOJRAJIVEE B, Nithish R, Loahith V</v>
       </c>
       <c r="G35" t="str">
-        <v>PS #10</v>
+        <v>PS #25</v>
       </c>
       <c r="H35" t="str">
-        <v>Catastrophe Risk Modelling</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="I35" t="str">
-        <v>ClimateTech &amp; Catastrophe Risk</v>
+        <v>Smart Mobility &amp; Usage-Based Insurance</v>
       </c>
       <c r="J35" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K35" t="str">
         <v>SY08 - Team JETG</v>
@@ -1693,13 +1693,13 @@
         <v>Shivasakthi R</v>
       </c>
       <c r="G37" t="str">
-        <v>PS #22</v>
+        <v>PS #17</v>
       </c>
       <c r="H37" t="str">
-        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
+        <v>Real-Time Indian Sign Language Translator</v>
       </c>
       <c r="I37" t="str">
-        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
+        <v>Computer Vision &amp; Accessibility (ISL)</v>
       </c>
       <c r="J37" t="str">
         <v>HARD</v>
@@ -1728,13 +1728,13 @@
         <v>Naveenkumar P, Mownaprasath R K, Nisanth P</v>
       </c>
       <c r="G38" t="str">
-        <v>PS #13</v>
+        <v>PS #18</v>
       </c>
       <c r="H38" t="str">
-        <v>Healthcare Interoperability</v>
+        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
       </c>
       <c r="I38" t="str">
-        <v>HealthTech &amp; FHIR Interoperability</v>
+        <v>LegalTech &amp; Contract Risk Copilot</v>
       </c>
       <c r="J38" t="str">
         <v>HARD</v>
@@ -1763,16 +1763,16 @@
         <v>Sivanesh.m, ELANGO S, Manoj .s</v>
       </c>
       <c r="G39" t="str">
-        <v>PS #27</v>
+        <v>PS #22</v>
       </c>
       <c r="H39" t="str">
-        <v>Multimodal AI Copilot for Accessibility &amp; Assistive Vision</v>
+        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
       </c>
       <c r="I39" t="str">
-        <v>Computer Vision &amp; Assistive AI</v>
+        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
       </c>
       <c r="J39" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K39" t="str">
         <v>SY12 - K4 boys</v>
@@ -1798,13 +1798,13 @@
         <v>A.Monish, M.Mohammaed Aflal Hussain, M.Kavin</v>
       </c>
       <c r="G40" t="str">
-        <v>PS #24</v>
+        <v>PS #14</v>
       </c>
       <c r="H40" t="str">
-        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
+        <v>Readmission Prevention</v>
       </c>
       <c r="I40" t="str">
-        <v>Digital Forensics &amp; Evidence Integrity</v>
+        <v>HealthTech &amp; Predictive AI</v>
       </c>
       <c r="J40" t="str">
         <v>HARD</v>
@@ -1833,16 +1833,16 @@
         <v>K.Mohammed Arshath, R.Logeshwar, P.Pranesh</v>
       </c>
       <c r="G41" t="str">
-        <v>PS #18</v>
+        <v>PS #09</v>
       </c>
       <c r="H41" t="str">
-        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
+        <v>Embedded Insurance</v>
       </c>
       <c r="I41" t="str">
-        <v>LegalTech &amp; Contract Risk Copilot</v>
+        <v>InsurTech &amp; Embedded Finance</v>
       </c>
       <c r="J41" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K41" t="str">
         <v>SY14 - NovaCrews</v>
@@ -1868,16 +1868,16 @@
         <v>Jayanthan p, Vijayaragavan A, Hemanth p</v>
       </c>
       <c r="G42" t="str">
-        <v>PS #11</v>
+        <v>PS #20</v>
       </c>
       <c r="H42" t="str">
-        <v>Prior Authorisation Automation</v>
+        <v>AI Grievance Redressal Prioritization System</v>
       </c>
       <c r="I42" t="str">
-        <v>HealthTech &amp; Prior Authorisation</v>
+        <v>GovTech &amp; Multilingual Grievance NLP</v>
       </c>
       <c r="J42" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K42" t="str">
         <v>SY15 - Logic Makers</v>
@@ -1903,13 +1903,13 @@
         <v>Saparna</v>
       </c>
       <c r="G43" t="str">
-        <v>PS #08</v>
+        <v>PS #12</v>
       </c>
       <c r="H43" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Clinical Documentation</v>
       </c>
       <c r="I43" t="str">
-        <v>InsurTech &amp; IoT Telematics</v>
+        <v>HealthTech &amp; Clinical Speech NLP</v>
       </c>
       <c r="J43" t="str">
         <v>MEDIUM</v>
@@ -1938,13 +1938,13 @@
         <v>S Nithyaasri, N Femina, M Priyadharshini</v>
       </c>
       <c r="G44" t="str">
-        <v>PS #12</v>
+        <v>PS #07</v>
       </c>
       <c r="H44" t="str">
-        <v>Clinical Documentation</v>
+        <v>End-to-End Claims Automation</v>
       </c>
       <c r="I44" t="str">
-        <v>HealthTech &amp; Clinical Speech NLP</v>
+        <v>InsurTech &amp; Claims Processing</v>
       </c>
       <c r="J44" t="str">
         <v>MEDIUM</v>
@@ -1973,16 +1973,16 @@
         <v>AKALYA S, HASINI E, DHANUJA B</v>
       </c>
       <c r="G45" t="str">
-        <v>PS #06</v>
+        <v>PS #03</v>
       </c>
       <c r="H45" t="str">
-        <v>Underwriting Automation</v>
+        <v>Personalised Banking</v>
       </c>
       <c r="I45" t="str">
-        <v>InsurTech &amp; Automated Underwriting</v>
+        <v>FinTech &amp; Personalization</v>
       </c>
       <c r="J45" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K45" t="str">
         <v>SY18 - Tech Vision</v>
@@ -2008,16 +2008,16 @@
         <v>P.M.Madhumita, D.Keerthana, S.Ponmalar</v>
       </c>
       <c r="G46" t="str">
-        <v>PS #26</v>
+        <v>PS #15</v>
       </c>
       <c r="H46" t="str">
-        <v>Autonomous Zero-Trust API Security &amp; Anomaly Shield</v>
+        <v>Value-Based Care Analytics</v>
       </c>
       <c r="I46" t="str">
-        <v>Cybersecurity &amp; Cloud Security</v>
+        <v>HealthTech &amp; Value-Based Analytics</v>
       </c>
       <c r="J46" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K46" t="str">
         <v>SY19 - SMIS</v>
@@ -2043,16 +2043,16 @@
         <v>Rithish, Ramji, Thilak</v>
       </c>
       <c r="G47" t="str">
-        <v>PS #20</v>
+        <v>PS #16</v>
       </c>
       <c r="H47" t="str">
-        <v>AI Grievance Redressal Prioritization System</v>
+        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
       </c>
       <c r="I47" t="str">
-        <v>GovTech &amp; Multilingual Grievance NLP</v>
+        <v>AI Mesh Networks &amp; Disaster Response</v>
       </c>
       <c r="J47" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K47" t="str">
         <v>SY20 - Team Electron</v>
@@ -2113,13 +2113,13 @@
         <v>Porkala</v>
       </c>
       <c r="G49" t="str">
-        <v>PS #19</v>
+        <v>PS #13</v>
       </c>
       <c r="H49" t="str">
-        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
+        <v>Healthcare Interoperability</v>
       </c>
       <c r="I49" t="str">
-        <v>Enterprise AI &amp; Multi-Source RAG</v>
+        <v>HealthTech &amp; FHIR Interoperability</v>
       </c>
       <c r="J49" t="str">
         <v>HARD</v>
@@ -2148,16 +2148,16 @@
         <v>PRADEEP P</v>
       </c>
       <c r="G50" t="str">
-        <v>PS #15</v>
+        <v>PS #06</v>
       </c>
       <c r="H50" t="str">
-        <v>Value-Based Care Analytics</v>
+        <v>Underwriting Automation</v>
       </c>
       <c r="I50" t="str">
-        <v>HealthTech &amp; Value-Based Analytics</v>
+        <v>InsurTech &amp; Automated Underwriting</v>
       </c>
       <c r="J50" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K50" t="str">
         <v>SY23 - AI Thinkers</v>
@@ -2183,19 +2183,19 @@
         <v>Selvakumarasamy S, Ragavan S, Vignesh S</v>
       </c>
       <c r="G51" t="str">
-        <v>PS #09</v>
+        <v>PS #01</v>
       </c>
       <c r="H51" t="str">
-        <v>Embedded Insurance</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="I51" t="str">
-        <v>InsurTech &amp; Embedded Finance</v>
+        <v>FinTech &amp; AI</v>
       </c>
       <c r="J51" t="str">
         <v>MEDIUM</v>
       </c>
       <c r="K51" t="str">
-        <v>SY24 - TECH SPARKZ</v>
+        <v>SY24 - TECH SPARKZ | SY26 - Phoenix | SY52 - Hack Fusion</v>
       </c>
     </row>
     <row r="52">
@@ -2218,16 +2218,16 @@
         <v>Dharshani T, Boomika KR, Abiramy S</v>
       </c>
       <c r="G52" t="str">
-        <v>PS #25</v>
+        <v>PS #11</v>
       </c>
       <c r="H52" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Prior Authorisation Automation</v>
       </c>
       <c r="I52" t="str">
-        <v>Smart Mobility &amp; Usage-Based Insurance</v>
+        <v>HealthTech &amp; Prior Authorisation</v>
       </c>
       <c r="J52" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K52" t="str">
         <v>SY25 - Zyntra</v>
@@ -2253,19 +2253,19 @@
         <v>N/A</v>
       </c>
       <c r="G53" t="str">
-        <v>PS #02</v>
+        <v>PS #01</v>
       </c>
       <c r="H53" t="str">
-        <v>Fraud Detection</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="I53" t="str">
-        <v>FinTech &amp; Cybersecurity</v>
+        <v>FinTech &amp; AI</v>
       </c>
       <c r="J53" t="str">
-        <v>HARD</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K53" t="str">
-        <v>SY26 - Phoenix</v>
+        <v>SY24 - TECH SPARKZ | SY26 - Phoenix | SY50 - Chaos coders</v>
       </c>
     </row>
     <row r="54">
@@ -2288,19 +2288,19 @@
         <v>N/A</v>
       </c>
       <c r="G54" t="str">
-        <v>PS #05</v>
+        <v>PS #24</v>
       </c>
       <c r="H54" t="str">
-        <v>Payments Modernisation</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="I54" t="str">
-        <v>Payments Modernisation</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
       <c r="J54" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K54" t="str">
-        <v>SY54 - Claude Busters</v>
+        <v>SY03 - BroVerse | SY29 - WhyNot | SY54 - Claude Busters</v>
       </c>
     </row>
     <row r="55">
@@ -2323,19 +2323,19 @@
         <v>N CAVIRAJ, P DINESH KUMAR, K AROKIA RAVIN</v>
       </c>
       <c r="G55" t="str">
-        <v>PS #05</v>
+        <v>PS #24</v>
       </c>
       <c r="H55" t="str">
-        <v>Payments Modernisation</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="I55" t="str">
-        <v>Payments Modernisation</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
       <c r="J55" t="str">
-        <v>MEDIUM</v>
+        <v>HARD</v>
       </c>
       <c r="K55" t="str">
-        <v>SY53 - Tech Titans</v>
+        <v>SY03 - BroVerse | SY29 - WhyNot | SY53 - Tech Titans</v>
       </c>
     </row>
     <row r="56">
@@ -2358,16 +2358,16 @@
         <v>Alex M, Sam K, Jordan P, Sam K, Alex M, Sam K, Jordan P, Jordan P, Alex M</v>
       </c>
       <c r="G56" t="str">
-        <v>PS #99</v>
+        <v>Unassigned</v>
       </c>
       <c r="H56" t="str">
-        <v>Synapse Developer Sandbox &amp; Integration Challenge</v>
+        <v>Unassigned</v>
       </c>
       <c r="I56" t="str">
-        <v>Platform Testing &amp; Sandbox</v>
+        <v>N/A</v>
       </c>
       <c r="J56" t="str">
-        <v>EASY</v>
+        <v>MEDIUM</v>
       </c>
       <c r="K56" t="str">
         <v>Test Team (Solo)</v>
@@ -2437,13 +2437,13 @@
         <v>VYOM</v>
       </c>
       <c r="F2" t="str">
-        <v>PS #16</v>
+        <v>PS #10</v>
       </c>
       <c r="G2" t="str">
-        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
+        <v>Catastrophe Risk Modelling</v>
       </c>
       <c r="H2" t="str">
-        <v>AI Mesh Networks &amp; Disaster Response</v>
+        <v>ClimateTech &amp; Catastrophe Risk</v>
       </c>
     </row>
     <row r="3">
@@ -2463,13 +2463,13 @@
         <v>TEAM PulseGuard</v>
       </c>
       <c r="F3" t="str">
-        <v>PS #04</v>
+        <v>PS #05</v>
       </c>
       <c r="G3" t="str">
-        <v>Open Banking &amp; APIs</v>
+        <v>Payments Modernisation</v>
       </c>
       <c r="H3" t="str">
-        <v>Open Banking &amp; API Ecosystems</v>
+        <v>Payments Modernisation</v>
       </c>
     </row>
     <row r="4">
@@ -2489,13 +2489,13 @@
         <v>WhyNot</v>
       </c>
       <c r="F4" t="str">
-        <v>PS #01</v>
+        <v>PS #24</v>
       </c>
       <c r="G4" t="str">
-        <v>Lending &amp; Credit</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="H4" t="str">
-        <v>FinTech &amp; AI</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
     </row>
     <row r="5">
@@ -2515,13 +2515,13 @@
         <v>SPARK SQUAD</v>
       </c>
       <c r="F5" t="str">
-        <v>PS #14</v>
+        <v>PS #02</v>
       </c>
       <c r="G5" t="str">
-        <v>Readmission Prevention</v>
+        <v>Fraud Detection</v>
       </c>
       <c r="H5" t="str">
-        <v>HealthTech &amp; Predictive AI</v>
+        <v>FinTech &amp; Cybersecurity</v>
       </c>
     </row>
     <row r="6">
@@ -2541,13 +2541,13 @@
         <v>Infinity loop</v>
       </c>
       <c r="F6" t="str">
-        <v>PS #17</v>
+        <v>PS #19</v>
       </c>
       <c r="G6" t="str">
-        <v>Real-Time Indian Sign Language Translator</v>
+        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
       </c>
       <c r="H6" t="str">
-        <v>Computer Vision &amp; Accessibility (ISL)</v>
+        <v>Enterprise AI &amp; Multi-Source RAG</v>
       </c>
     </row>
     <row r="7">
@@ -2567,13 +2567,13 @@
         <v>Elite-x</v>
       </c>
       <c r="F7" t="str">
-        <v>PS #03</v>
+        <v>PS #04</v>
       </c>
       <c r="G7" t="str">
-        <v>Personalised Banking</v>
+        <v>Open Banking &amp; APIs</v>
       </c>
       <c r="H7" t="str">
-        <v>FinTech &amp; Personalization</v>
+        <v>Open Banking &amp; API Ecosystems</v>
       </c>
     </row>
     <row r="8">
@@ -2593,13 +2593,13 @@
         <v>Brain bytes</v>
       </c>
       <c r="F8" t="str">
-        <v>PS #07</v>
+        <v>PS #08</v>
       </c>
       <c r="G8" t="str">
-        <v>End-to-End Claims Automation</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="H8" t="str">
-        <v>InsurTech &amp; Claims Processing</v>
+        <v>InsurTech &amp; IoT Telematics</v>
       </c>
     </row>
     <row r="9">
@@ -2619,13 +2619,13 @@
         <v>TECH NOVA</v>
       </c>
       <c r="F9" t="str">
-        <v>PS #10</v>
+        <v>PS #25</v>
       </c>
       <c r="G9" t="str">
-        <v>Catastrophe Risk Modelling</v>
+        <v>Usage-Based Insurance</v>
       </c>
       <c r="H9" t="str">
-        <v>ClimateTech &amp; Catastrophe Risk</v>
+        <v>Smart Mobility &amp; Usage-Based Insurance</v>
       </c>
     </row>
     <row r="10">
@@ -2671,13 +2671,13 @@
         <v>Think &amp; Sink</v>
       </c>
       <c r="F11" t="str">
-        <v>PS #22</v>
+        <v>PS #17</v>
       </c>
       <c r="G11" t="str">
-        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
+        <v>Real-Time Indian Sign Language Translator</v>
       </c>
       <c r="H11" t="str">
-        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
+        <v>Computer Vision &amp; Accessibility (ISL)</v>
       </c>
     </row>
     <row r="12">
@@ -2697,13 +2697,13 @@
         <v>Out of Memory</v>
       </c>
       <c r="F12" t="str">
-        <v>PS #13</v>
+        <v>PS #18</v>
       </c>
       <c r="G12" t="str">
-        <v>Healthcare Interoperability</v>
+        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
       </c>
       <c r="H12" t="str">
-        <v>HealthTech &amp; FHIR Interoperability</v>
+        <v>LegalTech &amp; Contract Risk Copilot</v>
       </c>
     </row>
     <row r="13">
@@ -2723,13 +2723,13 @@
         <v>AKATSUKI</v>
       </c>
       <c r="F13" t="str">
-        <v>PS #27</v>
+        <v>PS #22</v>
       </c>
       <c r="G13" t="str">
-        <v>Multimodal AI Copilot for Accessibility &amp; Assistive Vision</v>
+        <v>Decentralized Supply Chain Provenance for Pharmaceuticals</v>
       </c>
       <c r="H13" t="str">
-        <v>Computer Vision &amp; Assistive AI</v>
+        <v>Blockchain &amp; Pharmaceutical Supply Chain</v>
       </c>
     </row>
     <row r="14">
@@ -2749,13 +2749,13 @@
         <v>Mavericks</v>
       </c>
       <c r="F14" t="str">
-        <v>PS #24</v>
+        <v>PS #14</v>
       </c>
       <c r="G14" t="str">
-        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
+        <v>Readmission Prevention</v>
       </c>
       <c r="H14" t="str">
-        <v>Digital Forensics &amp; Evidence Integrity</v>
+        <v>HealthTech &amp; Predictive AI</v>
       </c>
     </row>
     <row r="15">
@@ -2775,13 +2775,13 @@
         <v>Code Creepers</v>
       </c>
       <c r="F15" t="str">
-        <v>PS #18</v>
+        <v>PS #09</v>
       </c>
       <c r="G15" t="str">
-        <v>Enterprise Legal Intelligence, Contract Risk &amp; Compliance Copilot</v>
+        <v>Embedded Insurance</v>
       </c>
       <c r="H15" t="str">
-        <v>LegalTech &amp; Contract Risk Copilot</v>
+        <v>InsurTech &amp; Embedded Finance</v>
       </c>
     </row>
     <row r="16">
@@ -2801,13 +2801,13 @@
         <v>Team Innovator's</v>
       </c>
       <c r="F16" t="str">
-        <v>PS #11</v>
+        <v>PS #20</v>
       </c>
       <c r="G16" t="str">
-        <v>Prior Authorisation Automation</v>
+        <v>AI Grievance Redressal Prioritization System</v>
       </c>
       <c r="H16" t="str">
-        <v>HealthTech &amp; Prior Authorisation</v>
+        <v>GovTech &amp; Multilingual Grievance NLP</v>
       </c>
     </row>
     <row r="17">
@@ -2827,13 +2827,13 @@
         <v>Nexus Neural</v>
       </c>
       <c r="F17" t="str">
-        <v>PS #08</v>
+        <v>PS #12</v>
       </c>
       <c r="G17" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Clinical Documentation</v>
       </c>
       <c r="H17" t="str">
-        <v>InsurTech &amp; IoT Telematics</v>
+        <v>HealthTech &amp; Clinical Speech NLP</v>
       </c>
     </row>
     <row r="18">
@@ -2853,13 +2853,13 @@
         <v>ZYRA</v>
       </c>
       <c r="F18" t="str">
-        <v>PS #12</v>
+        <v>PS #07</v>
       </c>
       <c r="G18" t="str">
-        <v>Clinical Documentation</v>
+        <v>End-to-End Claims Automation</v>
       </c>
       <c r="H18" t="str">
-        <v>HealthTech &amp; Clinical Speech NLP</v>
+        <v>InsurTech &amp; Claims Processing</v>
       </c>
     </row>
     <row r="19">
@@ -2879,13 +2879,13 @@
         <v>INNOVEXA</v>
       </c>
       <c r="F19" t="str">
-        <v>PS #06</v>
+        <v>PS #03</v>
       </c>
       <c r="G19" t="str">
-        <v>Underwriting Automation</v>
+        <v>Personalised Banking</v>
       </c>
       <c r="H19" t="str">
-        <v>InsurTech &amp; Automated Underwriting</v>
+        <v>FinTech &amp; Personalization</v>
       </c>
     </row>
     <row r="20">
@@ -2905,13 +2905,13 @@
         <v>Neura Nova</v>
       </c>
       <c r="F20" t="str">
-        <v>PS #26</v>
+        <v>PS #15</v>
       </c>
       <c r="G20" t="str">
-        <v>Autonomous Zero-Trust API Security &amp; Anomaly Shield</v>
+        <v>Value-Based Care Analytics</v>
       </c>
       <c r="H20" t="str">
-        <v>Cybersecurity &amp; Cloud Security</v>
+        <v>HealthTech &amp; Value-Based Analytics</v>
       </c>
     </row>
     <row r="21">
@@ -2931,13 +2931,13 @@
         <v>Hellfire</v>
       </c>
       <c r="F21" t="str">
-        <v>PS #20</v>
+        <v>PS #16</v>
       </c>
       <c r="G21" t="str">
-        <v>AI Grievance Redressal Prioritization System</v>
+        <v>Decentralized AI Agent Orchestrator for Disaster Response</v>
       </c>
       <c r="H21" t="str">
-        <v>GovTech &amp; Multilingual Grievance NLP</v>
+        <v>AI Mesh Networks &amp; Disaster Response</v>
       </c>
     </row>
     <row r="22">
@@ -2983,13 +2983,13 @@
         <v>Team Blossom</v>
       </c>
       <c r="F23" t="str">
-        <v>PS #19</v>
+        <v>PS #13</v>
       </c>
       <c r="G23" t="str">
-        <v>Enterprise Multi-Source RAG Intelligence &amp; Evidence Verification</v>
+        <v>Healthcare Interoperability</v>
       </c>
       <c r="H23" t="str">
-        <v>Enterprise AI &amp; Multi-Source RAG</v>
+        <v>HealthTech &amp; FHIR Interoperability</v>
       </c>
     </row>
     <row r="24">
@@ -3009,13 +3009,13 @@
         <v>AI Assist</v>
       </c>
       <c r="F24" t="str">
-        <v>PS #15</v>
+        <v>PS #06</v>
       </c>
       <c r="G24" t="str">
-        <v>Value-Based Care Analytics</v>
+        <v>Underwriting Automation</v>
       </c>
       <c r="H24" t="str">
-        <v>HealthTech &amp; Value-Based Analytics</v>
+        <v>InsurTech &amp; Automated Underwriting</v>
       </c>
     </row>
     <row r="25">
@@ -3029,19 +3029,19 @@
         <v>TECH SPARKZ</v>
       </c>
       <c r="D25" t="str">
-        <v>SY50</v>
+        <v>SY26</v>
       </c>
       <c r="E25" t="str">
-        <v>Chaos coders</v>
+        <v>Phoenix</v>
       </c>
       <c r="F25" t="str">
-        <v>PS #09</v>
+        <v>PS #01</v>
       </c>
       <c r="G25" t="str">
-        <v>Embedded Insurance</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="H25" t="str">
-        <v>InsurTech &amp; Embedded Finance</v>
+        <v>FinTech &amp; AI</v>
       </c>
     </row>
     <row r="26">
@@ -3061,13 +3061,13 @@
         <v>MindForge</v>
       </c>
       <c r="F26" t="str">
-        <v>PS #25</v>
+        <v>PS #11</v>
       </c>
       <c r="G26" t="str">
-        <v>Usage-Based Insurance</v>
+        <v>Prior Authorisation Automation</v>
       </c>
       <c r="H26" t="str">
-        <v>Smart Mobility &amp; Usage-Based Insurance</v>
+        <v>HealthTech &amp; Prior Authorisation</v>
       </c>
     </row>
     <row r="27">
@@ -3075,10 +3075,10 @@
         <v>Pair 26</v>
       </c>
       <c r="B27" t="str">
-        <v>SY26</v>
+        <v>SY50</v>
       </c>
       <c r="C27" t="str">
-        <v>Phoenix</v>
+        <v>Chaos coders</v>
       </c>
       <c r="D27" t="str">
         <v>SY52</v>
@@ -3087,13 +3087,13 @@
         <v>Hack Fusion</v>
       </c>
       <c r="F27" t="str">
-        <v>PS #02</v>
+        <v>PS #01</v>
       </c>
       <c r="G27" t="str">
-        <v>Fraud Detection</v>
+        <v>Lending &amp; Credit</v>
       </c>
       <c r="H27" t="str">
-        <v>FinTech &amp; Cybersecurity</v>
+        <v>FinTech &amp; AI</v>
       </c>
     </row>
     <row r="28">
@@ -3113,13 +3113,13 @@
         <v>Claude Busters</v>
       </c>
       <c r="F28" t="str">
-        <v>PS #05</v>
+        <v>PS #24</v>
       </c>
       <c r="G28" t="str">
-        <v>Payments Modernisation</v>
+        <v>AI-Powered Digital Evidence Integrity &amp; Fraud Investigation Platform</v>
       </c>
       <c r="H28" t="str">
-        <v>Payments Modernisation</v>
+        <v>Digital Forensics &amp; Evidence Integrity</v>
       </c>
     </row>
   </sheetData>

</xml_diff>